<commit_message>
Add weekly All Salons file(s) (06/20/2026)
</commit_message>
<xml_diff>
--- a/All Salons 06.19.26.xlsx
+++ b/All Salons 06.19.26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffd\OneDrive\Desktop\GC-Weekly-Stats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4EE9A9DC-4744-4363-893E-500C0EC8FAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD50F00-DAD7-4FCE-B776-3661D9ED0389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -554,6 +554,25 @@
   </cellStyles>
   <dxfs count="21">
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="165" formatCode="#,##0.0%;\-#,##0.0%;#,##0.0%"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -628,25 +647,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color auto="1"/>
@@ -667,31 +667,31 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D147E3D1-65A7-44D9-9298-7E5095024125}" name="Table1" displayName="Table1" ref="A1:S92" totalsRowShown="0" headerRowDxfId="19" headerRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D147E3D1-65A7-44D9-9298-7E5095024125}" name="Table1" displayName="Table1" ref="A1:S92" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="20">
   <autoFilter ref="A1:S92" xr:uid="{D147E3D1-65A7-44D9-9298-7E5095024125}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S92">
     <sortCondition descending="1" ref="E1:E92"/>
   </sortState>
   <tableColumns count="19">
-    <tableColumn id="1" xr3:uid="{56DDC4D4-518B-4FF0-8CCE-2DE66948BF68}" name="Salon" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{09ABB4BE-4E63-4B39-98D8-1020132FBBAC}" name="SalonWeekEndingDate" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{B0D74292-4335-4A38-82CB-3DB871DAD2B6}" name="Cust Count" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{55C8B665-52B2-4EBF-AA28-D379ACD4A83F}" name="Cust Count Last Year" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{BCEC69C5-231F-40A5-9727-6B440DDC1F32}" name="Cust Count % Change" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{B0F5AB79-40B9-4858-9B35-A5FEA15BC278}" name="New Cust" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{716C3B52-536D-44AC-BBC3-32376AA8419C}" name="New Cust %" dataDxfId="12"/>
-    <tableColumn id="8" xr3:uid="{D42FA9DA-1193-488F-884E-A6DD6BA4CDA5}" name="Salon New Cust Return %" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{B97030EB-2133-475E-8A88-B92F9ECBD47C}" name="Salon Repeat Cust Return %" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{A671ECA7-B615-4981-BFD5-548F871C0FA7}" name="Floor Hours" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{47FF8CD9-1AA1-432B-BA6C-453924111C20}" name="Sat/Sun Floor Hours %" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{4E47A839-9F2C-4E57-9144-00F0165C0981}" name="Floor Hours Growth" dataDxfId="7"/>
-    <tableColumn id="13" xr3:uid="{23B872AA-8257-474F-BFF2-6B282C69C540}" name="Wait Times &gt; 15Min %" dataDxfId="6"/>
-    <tableColumn id="14" xr3:uid="{5E53DFFA-56CC-4505-8EDB-2B58F05D0D3F}" name="Sat/Sun Wait Times &gt; 15Min %" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{8CC7C6E8-8EE5-44E1-9185-B442C3803FE5}" name="Avg Wait Time" dataDxfId="4"/>
-    <tableColumn id="16" xr3:uid="{8B16E5B4-ED4E-4207-A5FD-9CB68BBE0FE1}" name="Avg HC Time" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{A988F850-189C-4BBB-9BAE-CC7A59BAAC9D}" name="CPH" dataDxfId="2"/>
-    <tableColumn id="18" xr3:uid="{E09217F5-46F9-489D-91E3-BD471F6DFF66}" name="Productivity" dataDxfId="1"/>
-    <tableColumn id="19" xr3:uid="{A1CDD2B3-6AD8-4FB8-8DEA-E7E8F943562F}" name="Discount %" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{56DDC4D4-518B-4FF0-8CCE-2DE66948BF68}" name="Salon" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{09ABB4BE-4E63-4B39-98D8-1020132FBBAC}" name="SalonWeekEndingDate" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{B0D74292-4335-4A38-82CB-3DB871DAD2B6}" name="Cust Count" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{55C8B665-52B2-4EBF-AA28-D379ACD4A83F}" name="Cust Count Last Year" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{BCEC69C5-231F-40A5-9727-6B440DDC1F32}" name="Cust Count % Change" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{B0F5AB79-40B9-4858-9B35-A5FEA15BC278}" name="New Cust" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{716C3B52-536D-44AC-BBC3-32376AA8419C}" name="New Cust %" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{D42FA9DA-1193-488F-884E-A6DD6BA4CDA5}" name="Salon New Cust Return %" dataDxfId="12"/>
+    <tableColumn id="9" xr3:uid="{B97030EB-2133-475E-8A88-B92F9ECBD47C}" name="Salon Repeat Cust Return %" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{A671ECA7-B615-4981-BFD5-548F871C0FA7}" name="Floor Hours" dataDxfId="10"/>
+    <tableColumn id="11" xr3:uid="{47FF8CD9-1AA1-432B-BA6C-453924111C20}" name="Sat/Sun Floor Hours %" dataDxfId="9"/>
+    <tableColumn id="12" xr3:uid="{4E47A839-9F2C-4E57-9144-00F0165C0981}" name="Floor Hours Growth" dataDxfId="8"/>
+    <tableColumn id="13" xr3:uid="{23B872AA-8257-474F-BFF2-6B282C69C540}" name="Wait Times &gt; 15Min %" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{5E53DFFA-56CC-4505-8EDB-2B58F05D0D3F}" name="Sat/Sun Wait Times &gt; 15Min %" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{8CC7C6E8-8EE5-44E1-9185-B442C3803FE5}" name="Avg Wait Time" dataDxfId="5"/>
+    <tableColumn id="16" xr3:uid="{8B16E5B4-ED4E-4207-A5FD-9CB68BBE0FE1}" name="Avg HC Time" dataDxfId="4"/>
+    <tableColumn id="17" xr3:uid="{A988F850-189C-4BBB-9BAE-CC7A59BAAC9D}" name="CPH" dataDxfId="3"/>
+    <tableColumn id="18" xr3:uid="{E09217F5-46F9-489D-91E3-BD471F6DFF66}" name="Productivity" dataDxfId="2"/>
+    <tableColumn id="19" xr3:uid="{A1CDD2B3-6AD8-4FB8-8DEA-E7E8F943562F}" name="Discount %" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1018,7 +1018,13 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.7109375" customWidth="1"/>
-    <col min="2" max="19" width="21.85546875" style="12" customWidth="1"/>
+    <col min="2" max="6" width="21.85546875" style="12" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" style="12" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" style="12" customWidth="1"/>
+    <col min="9" max="9" width="18" style="12" customWidth="1"/>
+    <col min="10" max="10" width="21.85546875" style="12" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" style="12" customWidth="1"/>
+    <col min="12" max="19" width="21.85546875" style="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="4" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>